<commit_message>
update Minuswertung und Präsentation
</commit_message>
<xml_diff>
--- a/data/ergebnis.xlsx
+++ b/data/ergebnis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,12 +473,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1386271535</t>
+          <t>1015145957</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>rara; urheberrecht</t>
+          <t>archiv; bibliographie; museum</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -488,107 +488,103 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://d-nb.info/1386271535/04/text</t>
+          <t>https://d-nb.info/1015145957/04/text</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Der Bauprozess</t>
+          <t>"Ich bin mein Leben lang vom Glück verfolgt!"</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>prozessuale und materielle Probleme des zivilen Bauprozesses</t>
+          <t>Studien zu Leben und Werk des Steinbildhauers und Holzschnitzers Joseph Krautwald (1914 - 2003)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Werner, Ulrich</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Werner Verlag</t>
-        </is>
-      </c>
+          <t>Nießing, Melanie</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1392743419</t>
+          <t>1325160199</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>archiv; bookmark</t>
+          <t>archiv; bibliothek; illustration; landesbibliothek</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://d-nb.info/1392743419/04/text</t>
+          <t>https://d-nb.info/1325160199/04/text</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>It's (Im)possible formation: the Book</t>
+          <t>Was wäre Literatur +-x: Liechtenstein?</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Onomatopee Projects</t>
+          <t>Verlag Literaturhaus Liechtenstein</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1393219802</t>
+          <t>1371364222</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>illustrator; papier</t>
+          <t>alphabet; grafik; lexikon; urheberrecht</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://d-nb.info/1393219802/04/text</t>
+          <t>https://d-nb.info/1371364222/04/text</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>De boekenwereld</t>
+          <t>Starke Seiten - Medienbildung und Informatik</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Amsterdam University Press</t>
+          <t>Ernst Klett Verlag</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1396364412</t>
+          <t>1375160958</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bibliothek; handschrift; kupferstich; museum; schreiben; tapete; verlag</t>
+          <t>bibliothek; illustration; kinderbuchautor; lexikon; schreiben; vorlesen</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -598,73 +594,65 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://d-nb.info/1396364412/04/text</t>
+          <t>https://d-nb.info/1375160958/04/text</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Coburg - Gotha - 1826</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ein Herzog - zwei Residenzen : Begleitbuch zum 200. Jubiläum des Doppelherzogstums : Gotha - Coburg</t>
-        </is>
-      </c>
+          <t>ABC der Tiere</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Michael Imhof Verlag</t>
+          <t>Mildenberger</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1396365583</t>
+          <t>137516113X</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>wasserzeichen</t>
+          <t>bibliothek; illustration; kinderbuchautor; lexikon; schreiben; vorlesen</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://d-nb.info/1396365583/04/text</t>
+          <t>https://d-nb.info/137516113X/04/text</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Die digitale Inhaltsdokumentation der strafgerichtlichen Hauptverhandlung</t>
+          <t>ABC der Tiere</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Kranz, Patrick</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Nomos</t>
+          <t>Mildenberger</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1397005165</t>
+          <t>1378407288</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>bibliography; liturgica</t>
+          <t>buchhandlung</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -674,69 +662,909 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://d-nb.info/1397005165/04/text</t>
+          <t>https://d-nb.info/1378407288/04/text</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Encountering art</t>
+          <t>Sommerleuchten über der Freitagsbuchhandlung</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>theological approaches to visuality</t>
+          <t>Roman</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Knauß, Stefanie</t>
+          <t>Natori, Sawako</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Nomos</t>
+          <t>Piper</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1399207539</t>
+          <t>1382819722</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>atlas; buchdruck; drucker; grafik; verlag</t>
+          <t>plakat; schreiben; vorlesen</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1382819722/04/text</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>¿Qué pasa?</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>westermann</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1382823614</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>grafik; jugendbuch; schreiben</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1382823614/04/text</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>P.A.U.L. D.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>westermann</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>138293775X</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>bibliothek; jugendbibliothek; jugendliteratur; verleger</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/138293775X/04/text</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Jella Lepman</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>neue Perspektiven auf ihr Leben und Wirken</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>J.B. Metzler</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1384720278</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>alphabet; papier; schreiben</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1384720278/04/text</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Die steuerrechtlichen Kreis- und Rundschreiben des Bundes</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Kompaktsammlung der wichtigsten Verwaltungsverordnungen der Eidgenössischen Steuerverwaltung ESTV und der Schweizerischen Steuerkonferenz SSK : Ausgabe 2026</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Schweiz</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Verlag Steuern und Recht</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1387661523</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>bibliothek; schreiben; urheberrecht; verlag</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1387661523/04/text</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Compliance in Versicherungsunternehmen</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>rechtliche Anforderungen und praktische Umsetzung</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Bürkle, Jürgen</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>C.H. Beck</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1390717976</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>archiv; zensur; zensurfall</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1390717976/04/text</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Urbanes Kino</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>filmische Wirklichkeitsaneignungen und städtischer Wandel in New York, 1959-1966</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Hummel, Berit</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>transcript</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1390719278</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>papier; papierhandel</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1390719278/04/text</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Kapitalmarktrecht</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Buck-Heeb, Petra</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>C.F. Müller</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1391266862</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>archiv; papier; schreiben; signatur; sondersammlung; vorlesen</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://d-nb.info/1399207539/04/text</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Die 5. Revolution: KI + Roboter</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>wie Künstliche Intelligenz und Robotik unseren Alltag, unser Arbeitsleben und unsere Gesellschaft verändern</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Müller, Harald</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Verlag Diplomatic Council Publishing</t>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1391266862/04/text</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BeurkG mit NotAktVV und DONot</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Armbrüster, Christian</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Deutscher Notarverlag</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>139181245X</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>lesegeschichte</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/139181245X/04/text</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Die schönsten Sinnesspiele für Krippenkinder</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Wahrnehmungsideen für alle Jahreszeiten</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Bischoff, Marion</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Klett Kita</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1392209005</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>atlas; cliché</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1392209005/04/text</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L' héritage colonial du Maroc</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>actes du 8e Colloque maroco-allemand, Bayreuth 2011</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Naturwissenschaftliche Gesellschaft Bayreuth e.V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1393890369</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>satzverfahren; schreiben</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1393890369/04/text</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Einheitspatent und Einheitliches Patentgericht</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Hüttermann, Aloys</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Carl Heymanns Verlag</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1394119135</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>schreiben; signatur; urheberrecht</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1394119135/04/text</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Schweizerisches Vermessungsrecht</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>unter besonderer Berücksichtigung des Geoinformationsrechts und des Grundbuchrechts</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Huser, Meinrad</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Schulthess</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1397332182</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>druckgeschichte; handschrift; papier</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1397332182/04/text</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Goethes "Faust" - ein Lebenswerk</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ausgewählte Handschriften zur Entstehung</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Ludwig, Ariane</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Wallstein Verlag</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1402118090</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>illustration; mediengeschichte; schreiben; schriftsteller</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1402118090/04/text</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Abitur 2028 - Leistungsfach Deutsch</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>westermann</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1406087378</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>jugendbuch; papier; schreiben; vorlesen</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1406087378/04/text</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>P.A.U.L. D.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Westermann</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1406087505</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>karikatur; plakat; schreiben</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1406087505/04/text</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Mensch &amp; Politik Sekundarstufe I - Politik und Wirtschaft</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>westermann</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1412704960</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>alphabet; plakat; schreiben</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1412704960/04/text</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Prima aktiv</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Cornelsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1412708818</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>alphabet; grafik; schreiben; wandzeitung</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1412708818/04/text</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Prima aktiv</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Cornelsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1414638418</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>archiv; bibliothek; handschrift</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1414638418/04/text</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Clavierwerke</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Merula, Tarquinio</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>edition baroque</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1414638825</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>archiv; bibliothek; handschrift</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1414638825/04/text</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Clavierwerke</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Merula, Tarquinio</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>edition baroque</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1415537089</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ifla</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/1415537089/04/text</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Vertreibung ins Schlaraffenland</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Erzählungen, Berichte, Briefe</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Hanel, Bernd Michael</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Eigenverlag Bernd Michael Hanel</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>141598168X</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>papier; schreiben; schreiber</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/141598168X/04/text</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Das Buch für Männer, die einen Schritt voraus sind</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>101 verblüffende Fakten, erstaunliche Geschichten und clevere Quizfragen : das Geschenkbuch zum Staunen, Mitreden und Weitererzählen</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Ardenfels, Konstantin</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Markus Mägerle</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>999046322</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>bibliography; lecture</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://d-nb.info/999046322/04/text</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Under the radar</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>the first woman in radio astronomy: Ruby Payne-Scott</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Goss, W. M.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Springer</t>
         </is>
       </c>
     </row>

</xml_diff>